<commit_message>
fix: assign roster import ids by role
</commit_message>
<xml_diff>
--- a/web-admin-vue/public/templates/player-import-template.xlsx
+++ b/web-admin-vue/public/templates/player-import-template.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1087,7 +1087,14 @@
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
-          <t>5. 示例行可直接替换；如保留原示例，系统导入时会自动跳过</t>
+          <t>5. 工作人员（如领队/队医/主教练/助理教练）可不填球号和球场位置</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>6. 示例行可直接替换；如保留原示例，系统导入时会自动跳过</t>
         </is>
       </c>
     </row>

</xml_diff>